<commit_message>
sync: 2026-05-21 14:14:05 from Cowork
</commit_message>
<xml_diff>
--- a/outputs/Messenger_BuyerList_Valuation.xlsx
+++ b/outputs/Messenger_BuyerList_Valuation.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="822" uniqueCount="660">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="823" uniqueCount="661">
   <si>
     <t xml:space="preserve">Project Penumbra — Messenger Asset Sale</t>
   </si>
@@ -1612,6 +1612,9 @@
   </si>
   <si>
     <t xml:space="preserve">Adjusted replacement cost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Method 1 indicative value</t>
   </si>
   <si>
     <t xml:space="preserve">→ Method 1 result range:</t>
@@ -5858,21 +5861,20 @@
       <c r="C12" s="7" t="s">
         <v>518</v>
       </c>
-      <c r="D12" s="7" t="e">
-        <f aca="false">method 1 indicative value</f>
-        <v>#VALUE!</v>
+      <c r="D12" s="7" t="s">
+        <v>529</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="B14" s="31" t="n">
         <f aca="false">B12*0.75</f>
         <v>48600000</v>
       </c>
       <c r="C14" s="32" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="D14" s="31" t="n">
         <f aca="false">B12*1.25</f>
@@ -5881,26 +5883,26 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="B17" s="6" t="s">
         <v>410</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="B18" s="7" t="n">
         <v>2021</v>
@@ -5909,12 +5911,12 @@
         <v>75</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="B19" s="7" t="n">
         <v>2024</v>
@@ -5923,12 +5925,12 @@
         <v>125</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="B20" s="7" t="n">
         <v>2024</v>
@@ -5937,12 +5939,12 @@
         <v>22</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="B21" s="7" t="n">
         <v>2020</v>
@@ -5951,12 +5953,12 @@
         <v>45</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="B22" s="7" t="n">
         <v>2026</v>
@@ -5965,12 +5967,12 @@
         <v>55</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="B23" s="7" t="n">
         <v>2014</v>
@@ -5979,12 +5981,12 @@
         <v>90</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="B24" s="7" t="n">
         <v>2023</v>
@@ -5993,12 +5995,12 @@
         <v>50</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="C26" s="34" t="n">
         <f aca="false">MEDIAN(C18:C24)</f>
@@ -6007,7 +6009,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="C27" s="35" t="n">
         <f aca="false">C26*1.2</f>
@@ -6016,7 +6018,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="C28" s="35" t="n">
         <f aca="false">C27*0.75</f>
@@ -6025,7 +6027,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="C29" s="34" t="n">
         <f aca="false">C28</f>
@@ -6034,7 +6036,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6042,18 +6044,18 @@
         <v>22</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="B33" s="36" t="n">
         <v>0.4</v>
@@ -6063,12 +6065,12 @@
         <v>19.8</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="B34" s="36" t="n">
         <v>1</v>
@@ -6078,12 +6080,12 @@
         <v>49.5</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="7" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="B35" s="36" t="n">
         <v>1.4</v>
@@ -6093,12 +6095,12 @@
         <v>69.3</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="B36" s="36" t="n">
         <v>2.5</v>
@@ -6108,31 +6110,31 @@
         <v>123.75</v>
       </c>
       <c r="D36" s="7" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="6" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="38" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="B40" s="8" t="n">
         <v>40</v>
@@ -6146,7 +6148,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="38" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="B41" s="8" t="n">
         <v>30</v>
@@ -6160,7 +6162,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="38" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="B42" s="8" t="n">
         <v>20</v>
@@ -6174,7 +6176,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="38" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="B43" s="8" t="n">
         <v>30</v>
@@ -6188,7 +6190,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="39" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="B44" s="40" t="n">
         <v>45</v>
@@ -6230,7 +6232,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -6239,173 +6241,173 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="41" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="B4" s="41" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="41" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="B5" s="41" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="41" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="B6" s="41" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="41" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="B7" s="41" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="41" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="B8" s="41" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="41" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="B9" s="41" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="B12" s="26" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="C12" s="26"/>
       <c r="D12" s="26"/>
     </row>
     <row r="13" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="B13" s="26" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="C13" s="26"/>
       <c r="D13" s="26"/>
     </row>
     <row r="14" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="B14" s="26" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="C14" s="26"/>
       <c r="D14" s="26"/>
     </row>
     <row r="15" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="B15" s="26" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="C15" s="26"/>
       <c r="D15" s="26"/>
     </row>
     <row r="16" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="B16" s="26" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="C16" s="26"/>
       <c r="D16" s="26"/>
     </row>
     <row r="17" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="B17" s="26" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="C17" s="26"/>
       <c r="D17" s="26"/>
     </row>
     <row r="18" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="B18" s="26" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="C18" s="26"/>
       <c r="D18" s="26"/>
@@ -6446,7 +6448,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -6456,208 +6458,208 @@
         <v>98</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="42" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="C4" s="43" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="42" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="C5" s="43" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="42" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="C6" s="43" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="42" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="C7" s="43" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="42" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="C8" s="43" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="42" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="C9" s="43" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="42" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="C10" s="43" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="42" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="C11" s="43" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="42" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="C12" s="43" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="42" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="C13" s="43" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="42" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="C14" s="43" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="42" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="C15" s="43" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="42" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="C16" s="43" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="42" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="C17" s="43" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="42" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="C18" s="43" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="42" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="C19" s="43" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="42" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="C20" s="43" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="42" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="C21" s="43" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
     </row>
   </sheetData>

</xml_diff>